<commit_message>
Add Plastic colours repoort
</commit_message>
<xml_diff>
--- a/Plastic colours/Kolory plastiku.xlsx
+++ b/Plastic colours/Kolory plastiku.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nowystylglobal-my.sharepoint.com/personal/lukasz_wojcik_nowystyl_com/Documents/Dokumenty/GitHub/NS-PBI/Plastic colours/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{20C2710B-E039-49D5-B920-925DE8FF8708}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="55" documentId="8_{20C2710B-E039-49D5-B920-925DE8FF8708}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ECEABD51-2678-4BDB-887A-38A94AA538C1}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4A39ADBC-37A8-4E29-96B4-F12D07E7D592}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
+    <sheet name="Arkusz2" sheetId="5" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="20">
   <si>
     <t>Sitari</t>
   </si>
@@ -150,12 +151,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
@@ -490,7 +492,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53D6C3BB-D964-4CB6-AB20-1D0957511700}">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.85546875" customWidth="1"/>
@@ -498,280 +500,791 @@
     <col min="3" max="3" width="13.85546875" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="1">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="1">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="1">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="1">
+        <v>12273</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="1">
+        <v>1752</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11" s="1">
+        <v>42224</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" s="1">
+        <v>3077</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" s="1">
+        <v>6358</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="1">
+        <v>3683</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="1">
+        <v>4</v>
+      </c>
+      <c r="G16" s="4"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C17" s="1">
+        <v>1</v>
+      </c>
+      <c r="G17" s="4"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B18" t="s">
+        <v>3</v>
+      </c>
+      <c r="C18" s="1">
+        <v>37944</v>
+      </c>
+      <c r="G18" s="4"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" s="1">
+        <v>1538</v>
+      </c>
+      <c r="G19" s="4"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" s="1">
+        <v>493</v>
+      </c>
+      <c r="G20" s="4"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B21" t="s">
+        <v>1</v>
+      </c>
+      <c r="C21" s="1">
+        <v>4338</v>
+      </c>
+      <c r="G21" s="4"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B22" t="s">
+        <v>3</v>
+      </c>
+      <c r="C22" s="1">
+        <v>48972</v>
+      </c>
+      <c r="G22" s="4"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C23" s="1">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B24" t="s">
+        <v>1</v>
+      </c>
+      <c r="C24" s="1">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B25" t="s">
+        <v>14</v>
+      </c>
+      <c r="C25" s="1">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B26" t="s">
+        <v>15</v>
+      </c>
+      <c r="C26" s="1">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>13</v>
+      </c>
+      <c r="B27" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" s="1">
+        <v>1325</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2819026-7E61-4B89-9E6C-3F1BB79130BD}">
+  <dimension ref="A1:C46"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="21.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2">
-        <v>32</v>
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1">
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="1" t="s">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="1">
         <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="2">
-        <v>212</v>
+      <c r="A4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B5" s="1" t="s">
+      <c r="A5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="1">
         <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B6" s="1" t="s">
+      <c r="A6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="1">
+        <v>2679</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="1">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11" s="1">
+        <v>1309</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" s="1">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13" s="1">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="1">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" s="1">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>12</v>
+      </c>
+      <c r="B18" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18" s="1">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" t="s">
+        <v>3</v>
+      </c>
+      <c r="C19" s="1">
+        <v>5764</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20" t="s">
+        <v>1</v>
+      </c>
+      <c r="C20" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>13</v>
+      </c>
+      <c r="B21" t="s">
+        <v>14</v>
+      </c>
+      <c r="C21" s="1">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>13</v>
+      </c>
+      <c r="B22" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" s="1">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>13</v>
+      </c>
+      <c r="B23" t="s">
+        <v>16</v>
+      </c>
+      <c r="C23" s="1">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>0</v>
+      </c>
+      <c r="B24" t="s">
+        <v>1</v>
+      </c>
+      <c r="C24" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>0</v>
+      </c>
+      <c r="B25" t="s">
+        <v>3</v>
+      </c>
+      <c r="C25" s="1">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>0</v>
+      </c>
+      <c r="B26" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C26" s="1">
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B7" s="1" t="s">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>0</v>
+      </c>
+      <c r="B27" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="2">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+      <c r="C27" s="1">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C8" s="2">
-        <v>12273</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+      <c r="C28" s="1">
         <v>7</v>
       </c>
-      <c r="B9" s="1" t="s">
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>7</v>
+      </c>
+      <c r="B29" t="s">
+        <v>3</v>
+      </c>
+      <c r="C29" s="1">
+        <v>9594</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>7</v>
+      </c>
+      <c r="B30" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="2">
-        <v>1752</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B10" s="1"/>
-      <c r="C10" s="2">
+      <c r="C30" s="1">
+        <v>1154</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>9</v>
+      </c>
+      <c r="B31" t="s">
+        <v>3</v>
+      </c>
+      <c r="C31" s="1">
+        <v>40915</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>9</v>
+      </c>
+      <c r="B32" t="s">
+        <v>8</v>
+      </c>
+      <c r="C32" s="1">
+        <v>3031</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>10</v>
+      </c>
+      <c r="C33" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>10</v>
+      </c>
+      <c r="B34" t="s">
+        <v>3</v>
+      </c>
+      <c r="C34" s="1">
+        <v>5736</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>10</v>
+      </c>
+      <c r="B35" t="s">
+        <v>8</v>
+      </c>
+      <c r="C35" s="1">
+        <v>3534</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>11</v>
+      </c>
+      <c r="C36" s="1">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>11</v>
+      </c>
+      <c r="B37" t="s">
+        <v>1</v>
+      </c>
+      <c r="C37" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>11</v>
+      </c>
+      <c r="B38" t="s">
+        <v>3</v>
+      </c>
+      <c r="C38" s="1">
+        <v>37878</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>11</v>
+      </c>
+      <c r="B39" t="s">
+        <v>8</v>
+      </c>
+      <c r="C39" s="1">
+        <v>1537</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C11" s="2">
-        <v>42224</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12" s="2">
-        <v>3151</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" s="1"/>
-      <c r="C13" s="2">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C14" s="2">
-        <v>6358</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C15" s="2">
-        <v>3683</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B16" s="1"/>
-      <c r="C16" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C17" s="2">
-        <v>30253</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C18" s="2">
-        <v>6382</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B19" s="1"/>
-      <c r="C19" s="2">
-        <v>3344</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
+      <c r="C40" s="1">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>12</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C20" s="2">
-        <v>4338</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
+      <c r="B41" t="s">
+        <v>1</v>
+      </c>
+      <c r="C41" s="1">
+        <v>4118</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>12</v>
       </c>
-      <c r="B21" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C21" s="2">
-        <v>48874</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B22" s="1"/>
-      <c r="C22" s="2">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
+      <c r="B42" t="s">
+        <v>3</v>
+      </c>
+      <c r="C42" s="1">
+        <v>43208</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C23" s="2">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
+      <c r="B43" t="s">
+        <v>1</v>
+      </c>
+      <c r="C43" s="1">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>13</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B44" t="s">
         <v>14</v>
       </c>
-      <c r="C24" s="2">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
+      <c r="C44" s="1">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B45" t="s">
         <v>15</v>
       </c>
-      <c r="C25" s="2">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
+      <c r="C45" s="1">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>13</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B46" t="s">
         <v>16</v>
       </c>
-      <c r="C26" s="2">
-        <v>1325</v>
+      <c r="C46" s="1">
+        <v>1150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>